<commit_message>
fix: add code file
</commit_message>
<xml_diff>
--- a/pdb_itasser.xlsx
+++ b/pdb_itasser.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luho/Documents/GitHub/De-nevo-protein-3D-structure-yeast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F6EFC6D-0DFC-CA4C-A22F-73C147309D64}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05A91ACE-F6E3-5C49-9857-5CDE9CC5331C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35820" yWindow="560" windowWidth="28800" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36060" yWindow="3860" windowWidth="28800" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
     <t>{'#model': 'Model1:', ' C-score': '0.63', 'TM-score': '0.80+-0.09', 'RMSD(in Angstroms)': '5.9+-3.7'}</t>
   </si>
   <si>
-    <t>YCL040W@model1.pdb</t>
+    <t>YCL040W@model1</t>
   </si>
   <si>
     <t>YDL021W</t>
@@ -76,7 +76,7 @@
     <t>{'Name': 'Model1:', 'C-score': '-0.46', 'Exp.TM-Score': '0.65+-0.13', 'Exp.RMSD': '7.3+-4.2', 'No.of decoys': '7098', 'Cluster density': '0.1714'}</t>
   </si>
   <si>
-    <t>YDL021W@model1.pdb</t>
+    <t>YDL021W@model1</t>
   </si>
   <si>
     <t>YMR278W</t>
@@ -85,7 +85,7 @@
     <t>{'Name': 'Model1:', 'C-score': '-0.35', 'Exp.TM-Score': '0.67+-0.13', 'Exp.RMSD': '8.6+-4.5', 'No.of decoys': '2091', 'Cluster density': '0.1760'}</t>
   </si>
   <si>
-    <t>YMR278W@model1.pdb</t>
+    <t>YMR278W@model1</t>
   </si>
   <si>
     <t>YOL056W</t>
@@ -94,7 +94,7 @@
     <t>{'Name': 'Model1:', 'C-score': '-0.45', 'Exp.TM-Score': '0.66+-0.13', 'Exp.RMSD': '7.2+-4.2', 'No.of decoys': '7010', 'Cluster density': '0.1758'}</t>
   </si>
   <si>
-    <t>YOL056W@model1.pdb</t>
+    <t>YOL056W@model1</t>
   </si>
   <si>
     <t>YLR164W</t>
@@ -109,7 +109,7 @@
     <t>{'Name': 'Model1:', 'C-score': '-1.60', 'Exp.TM-Score': '0.52+-0.15', 'Exp.RMSD': '8.5+-4.5', 'No.of decoys': '3404', 'Cluster density': '0.0593'}</t>
   </si>
   <si>
-    <t>YLR164W@model1.pdb</t>
+    <t>YLR164W@model1</t>
   </si>
   <si>
     <t>YCR036W</t>
@@ -124,7 +124,7 @@
     <t>{'Name': 'Model1:', 'C-score': '0.53', 'Exp.TM-Score': '0.78+-0.09', 'Exp.RMSD': '5.3+-3.4', 'No.of decoys': '8035', 'Cluster density': '0.4501'}</t>
   </si>
   <si>
-    <t>YCR036W@model1.pdb</t>
+    <t>YCR036W@model1</t>
   </si>
   <si>
     <t>YCR073W-A</t>
@@ -133,7 +133,7 @@
     <t>{'Name': 'Model1:', 'C-score': '-1.06', 'Exp.TM-Score': '0.58+-0.14', 'Exp.RMSD': '8.7+-4.5', 'No.of decoys': '5398', 'Cluster density': '0.1036'}</t>
   </si>
   <si>
-    <t>YCR073W-A@model1.pdb</t>
+    <t>YCR073W-A@model1</t>
   </si>
   <si>
     <t>YKL181W</t>
@@ -142,7 +142,7 @@
     <t>{'Name': 'Model1:', 'C-score': '-1.66', 'Exp.TM-Score': '0.51+-0.15', 'Exp.RMSD': '10.8+-4.6', 'No.of decoys': '734', 'Cluster density': '0.0423'}</t>
   </si>
   <si>
-    <t>YKL181W@model1.pdb</t>
+    <t>YKL181W@model1</t>
   </si>
   <si>
     <t>YNR034W</t>
@@ -151,7 +151,7 @@
     <t>{'#model': 'Model1:', ' C-score': '-0.98', 'TM-score': '0.59+-0.14', 'RMSD(in Angstroms)': '8.5+-4.5'}</t>
   </si>
   <si>
-    <t>YNR034W@model1.pdb</t>
+    <t>YNR034W@model1</t>
   </si>
   <si>
     <t>YDR322C-A</t>
@@ -166,7 +166,7 @@
     <t>{'Name': 'Model1:', 'C-score': '-3.13', 'Exp.TM-Score': '0.36+-0.12', 'Exp.RMSD': '10.8+-4.6', 'No.of decoys': '1963', 'Cluster density': '0.0691'}</t>
   </si>
   <si>
-    <t>YDR322C-A@model1.pdb</t>
+    <t>YDR322C-A@model1</t>
   </si>
   <si>
     <t>YER141W</t>
@@ -175,7 +175,7 @@
     <t>{'Name': 'Model1:', 'C-score': '-0.17', 'Exp.TM-Score': '0.69+-0.12', 'Exp.RMSD': '7.6+-4.3', 'No.of decoys': '600', 'Cluster density': '0.2083'}</t>
   </si>
   <si>
-    <t>YER141W@model1.pdb</t>
+    <t>YER141W@model1</t>
   </si>
   <si>
     <t>YGL008C</t>
@@ -184,7 +184,7 @@
     <t>{'Name': 'Model1:', 'C-score': '2.00', 'Exp.TM-Score': '0.99+-0.04', 'Exp.RMSD': '4.0+-2.7', 'No.of decoys': '3000', 'Cluster density': '1.2500'}</t>
   </si>
   <si>
-    <t>YGL008C@model1.pdb</t>
+    <t>YGL008C@model1</t>
   </si>
   <si>
     <t>YPL036W</t>
@@ -193,7 +193,7 @@
     <t>{'Name': 'Model1:', 'C-score': '1.21', 'Exp.TM-Score': '0.88+-0.07', 'Exp.RMSD': '6.1+-3.7', 'No.of decoys': '2347', 'Cluster density': '0.4054'}</t>
   </si>
   <si>
-    <t>YPL036W@model1.pdb</t>
+    <t>YPL036W@model1</t>
   </si>
   <si>
     <t>YPL132W</t>
@@ -202,7 +202,7 @@
     <t>{'#model': 'Model1:', ' C-score': '-3.86', 'TM-score': '0.30+-0.10', 'RMSD(in Angstroms)': '15.7+-3.3'}</t>
   </si>
   <si>
-    <t>YPL132W@model1.pdb</t>
+    <t>YPL132W@model1</t>
   </si>
   <si>
     <t>YPL172C</t>
@@ -211,7 +211,7 @@
     <t>{'Name': 'Model1:', 'C-score': '-0.90', 'Exp.TM-Score': '0.60+-0.14', 'Exp.RMSD': '9.2+-4.6', 'No.of decoys': '600', 'Cluster density': '0.1156'}</t>
   </si>
   <si>
-    <t>YPL172C@model1.pdb</t>
+    <t>YPL172C@model1</t>
   </si>
   <si>
     <t>YPR020W</t>
@@ -220,7 +220,7 @@
     <t>{'Name': 'Model1:', 'C-score': '-3.36', 'Exp.TM-Score': '0.34+-0.11', 'Exp.RMSD': '11.8+-4.5', 'No.of decoys': '1850', 'Cluster density': '0.0562'}</t>
   </si>
   <si>
-    <t>YPR020W@model1.pdb</t>
+    <t>YPR020W@model1</t>
   </si>
 </sst>
 </file>
@@ -276,11 +276,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -587,606 +586,599 @@
   <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="3" width="8.83203125" style="1"/>
-    <col min="4" max="4" width="25.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="112.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="25" style="1" customWidth="1"/>
-    <col min="8" max="8" width="23.5" style="1" customWidth="1"/>
-    <col min="9" max="9" width="8.83203125" style="1"/>
-    <col min="10" max="10" width="19" style="1" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="48.1640625" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2">
         <v>500</v>
       </c>
-      <c r="I2" s="1">
-        <v>1</v>
-      </c>
-      <c r="J2" s="1">
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
         <v>500</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3">
         <v>311</v>
       </c>
-      <c r="I3" s="1">
-        <v>1</v>
-      </c>
-      <c r="J3" s="1">
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
         <v>311</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4">
         <v>622</v>
       </c>
-      <c r="I4" s="1">
-        <v>1</v>
-      </c>
-      <c r="J4" s="1">
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
         <v>622</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="1" t="s">
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
         <v>23</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" t="s">
         <v>24</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5">
         <v>303</v>
       </c>
-      <c r="I5" s="1">
-        <v>1</v>
-      </c>
-      <c r="J5" s="1">
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
         <v>303</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="1" t="s">
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
         <v>28</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" t="s">
         <v>29</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6">
         <v>168</v>
       </c>
-      <c r="I6" s="1">
-        <v>1</v>
-      </c>
-      <c r="J6" s="1">
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
         <v>168</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="K6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="1" t="s">
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" t="s">
         <v>34</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7">
         <v>333</v>
       </c>
-      <c r="I7" s="1">
-        <v>1</v>
-      </c>
-      <c r="J7" s="1">
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
         <v>333</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="K7" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="1" t="s">
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
         <v>36</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" t="s">
         <v>37</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8">
         <v>315</v>
       </c>
-      <c r="I8" s="1">
-        <v>1</v>
-      </c>
-      <c r="J8" s="1">
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
         <v>315</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="K8" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" t="s">
         <v>32</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="1" t="s">
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" t="s">
         <v>40</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9">
         <v>427</v>
       </c>
-      <c r="I9" s="1">
-        <v>1</v>
-      </c>
-      <c r="J9" s="1">
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
         <v>427</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="K9" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="1" t="s">
+      <c r="E10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" t="s">
         <v>42</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" t="s">
         <v>43</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10">
         <v>321</v>
       </c>
-      <c r="I10" s="1">
-        <v>1</v>
-      </c>
-      <c r="J10" s="1">
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10">
         <v>321</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="K10" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>37</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="1" t="s">
+      <c r="E11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" t="s">
         <v>47</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" t="s">
         <v>48</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11">
         <v>96</v>
       </c>
-      <c r="I11" s="1">
-        <v>1</v>
-      </c>
-      <c r="J11" s="1">
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="J11">
         <v>96</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="K11" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>38</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="1" t="s">
+      <c r="E12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s">
         <v>50</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="G12" t="s">
         <v>51</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12">
         <v>486</v>
       </c>
-      <c r="I12" s="1">
-        <v>1</v>
-      </c>
-      <c r="J12" s="1">
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="J12">
         <v>486</v>
       </c>
-      <c r="K12" s="1" t="s">
+      <c r="K12" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>39</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="1" t="s">
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s">
         <v>53</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="G13" t="s">
         <v>54</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13">
         <v>918</v>
       </c>
-      <c r="I13" s="1">
-        <v>1</v>
-      </c>
-      <c r="J13" s="1">
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13">
         <v>918</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="K13" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>40</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" t="s">
         <v>46</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="1" t="s">
+      <c r="E14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s">
         <v>56</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="G14" t="s">
         <v>57</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14">
         <v>947</v>
       </c>
-      <c r="I14" s="1">
-        <v>1</v>
-      </c>
-      <c r="J14" s="1">
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14">
         <v>947</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="K14" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>41</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>58</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="1" t="s">
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
         <v>59</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="G15" t="s">
         <v>60</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15">
         <v>300</v>
       </c>
-      <c r="I15" s="1">
-        <v>1</v>
-      </c>
-      <c r="J15" s="1">
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15">
         <v>300</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="K15" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>42</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" s="1" t="s">
+      <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s">
         <v>62</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="G16" t="s">
         <v>63</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16">
         <v>462</v>
       </c>
-      <c r="I16" s="1">
-        <v>1</v>
-      </c>
-      <c r="J16" s="1">
+      <c r="I16">
+        <v>1</v>
+      </c>
+      <c r="J16">
         <v>462</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="K16" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>43</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>64</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F17" s="1" t="s">
+      <c r="E17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" t="s">
         <v>65</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="G17" t="s">
         <v>66</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17">
         <v>115</v>
       </c>
-      <c r="I17" s="1">
-        <v>1</v>
-      </c>
-      <c r="J17" s="1">
+      <c r="I17">
+        <v>1</v>
+      </c>
+      <c r="J17">
         <v>115</v>
       </c>
-      <c r="K17" s="1" t="s">
+      <c r="K17" t="s">
         <v>64</v>
       </c>
     </row>

</xml_diff>